<commit_message>
Update BRD and remove per-customer Excel exports from tracking
- BRD_and_TestCases.docx regenerated with latest content
- Delete CUST0009/0010/0012/0030.xlsx — now covered by .gitignore
  (regenerable via solution_code/customer_360.py)
- CUST0013.xlsx kept as a sample/demo of the 360 export format
</commit_message>
<xml_diff>
--- a/CUST0013.xlsx
+++ b/CUST0013.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Customer" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Vehicle" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Service" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Insurance" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Churn_Features" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Churn_Score" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PII_Vault" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Vehicle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sales" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Service" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Insurance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Churn_Features" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Churn_Score" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -155,6 +161,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,6 +904,169 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>PII VAULT (Raw — Authorised Access)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>cust_id</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>cust_name</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>mobile_1</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>mobile_2</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>dob</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>pincode</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>occ_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CUST0013</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Arun Pillai</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>6143634957</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>8685574443</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>arun.pillai22@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>20-07-1971</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>16, Park Street, Chennai</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>600040</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>OCC004</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -917,84 +1092,84 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>VEHICLE(S) OWNED</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>vehicle_id</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>vin</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>reg_no</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>engine_no</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>variant</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>color</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>cc</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>mfd_year</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="10" t="inlineStr">
         <is>
           <t>registration_date</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="10" t="inlineStr">
         <is>
           <t>fuel_type_id</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="10" t="inlineStr">
         <is>
           <t>transmission</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="10" t="inlineStr">
         <is>
           <t>body_type</t>
         </is>
       </c>
-      <c r="N2" s="8" t="inlineStr">
+      <c r="N2" s="10" t="inlineStr">
         <is>
           <t>seating_capacity</t>
         </is>
       </c>
-      <c r="O2" s="8" t="inlineStr">
+      <c r="O2" s="10" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
@@ -1079,7 +1254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -1106,79 +1281,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>SALES TRANSACTIONS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>sales_id</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>cust_id</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>dealer_id</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>vin</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>mfd_year</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>registration_date</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>tax_validity</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>pucc_validity</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>finance_flag</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>bank_id</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>sale_date</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
       </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>sales_poc</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>loc_id</t>
         </is>
@@ -1258,7 +1433,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -1285,79 +1460,79 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>SERVICE HISTORY</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>smr_id</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>cust_id</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>dealer_id</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>vin</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>work_type_id</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>milestone_id</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>visit_date</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>bill_date</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>cancel_reason_id</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>bill_amount</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>mileage</t>
         </is>
       </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>service_advisor</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>pay_mode_id</t>
         </is>
@@ -1563,7 +1738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -1591,84 +1766,84 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>INSURANCE HISTORY</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>ins_id</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>cust_id</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>dealer_id</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>vin</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>policy_type_id</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>policy_no</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>policy_issue_date</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>policy_inception_date</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>policy_expiry_date</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>tp_policy_issue_date</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>tp_policy_expiry_date</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>previous_policy_start_date</t>
         </is>
       </c>
-      <c r="M2" s="10" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>previous_policy_end_date</t>
         </is>
       </c>
-      <c r="N2" s="10" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>auto_membership</t>
         </is>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="O2" s="12" t="inlineStr">
         <is>
           <t>total_premium</t>
         </is>
@@ -1749,7 +1924,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -1781,104 +1956,104 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>CHURN FEATURES (Engineered)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>cust_id</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>vehicle_id</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>vehicle_age_years</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>finance_flag</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>total_service_visits</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>days_since_last_service</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>avg_bill_amount</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>pct_paid_services</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="14" t="inlineStr">
         <is>
           <t>cancelled_visit_flag</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="14" t="inlineStr">
         <is>
           <t>num_policy_renewals</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="14" t="inlineStr">
         <is>
           <t>days_to_policy_expiry</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="14" t="inlineStr">
         <is>
           <t>auto_membership_flag</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="14" t="inlineStr">
         <is>
           <t>premium_trend</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="14" t="inlineStr">
         <is>
           <t>recency_score</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="14" t="inlineStr">
         <is>
           <t>frequency_score</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="14" t="inlineStr">
         <is>
           <t>monetary_score</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="14" t="inlineStr">
         <is>
           <t>rfm_total</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr">
+      <c r="R2" s="14" t="inlineStr">
         <is>
           <t>churn_label</t>
         </is>
       </c>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="S2" s="14" t="inlineStr">
         <is>
           <t>risk_tier</t>
         </is>
@@ -1959,7 +2134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -1980,49 +2155,49 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>CHURN SCORE &amp; RECOMMENDED ACTION</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>cust_id</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>churn_probability</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>risk_tier</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>top_driver_1</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>top_driver_2</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>top_driver_3</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>recommended_action</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>score_date</t>
         </is>

</xml_diff>